<commit_message>
update qc to fill in missing values
</commit_message>
<xml_diff>
--- a/qc/spreadsheets/sharedreward_qc.xlsx
+++ b/qc/spreadsheets/sharedreward_qc.xlsx
@@ -11,7 +11,7 @@
     <sheet name="thresholds" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'runs'!$A$1:$Y$664</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'runs'!$A$1:$Y$666</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'thresholds'!$A$1:$K$5</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y664"/>
+  <dimension ref="A1:Y666"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -464,8 +464,8 @@
     <col width="20" customWidth="1" min="17" max="17"/>
     <col width="45" customWidth="1" min="18" max="18"/>
     <col width="13" customWidth="1" min="19" max="19"/>
-    <col width="45" customWidth="1" min="20" max="20"/>
-    <col width="12" customWidth="1" min="21" max="21"/>
+    <col width="17" customWidth="1" min="20" max="20"/>
+    <col width="11" customWidth="1" min="21" max="21"/>
     <col width="45" customWidth="1" min="22" max="22"/>
     <col width="45" customWidth="1" min="23" max="23"/>
     <col width="45" customWidth="1" min="24" max="24"/>
@@ -17041,26 +17041,42 @@
       <c r="G182" t="n">
         <v>0.1861611225688447</v>
       </c>
+      <c r="H182" t="n">
+        <v>20</v>
+      </c>
+      <c r="I182" t="n">
+        <v>11</v>
+      </c>
+      <c r="J182" t="n">
+        <v>9</v>
+      </c>
+      <c r="K182" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="L182" t="n">
+        <v>99.98538710877305</v>
+      </c>
       <c r="M182" t="b">
         <v>0</v>
       </c>
       <c r="N182" t="b">
         <v>0</v>
       </c>
+      <c r="O182" t="b">
+        <v>0</v>
+      </c>
+      <c r="P182" t="b">
+        <v>0</v>
+      </c>
       <c r="Q182" t="b">
         <v>0</v>
       </c>
       <c r="S182" t="b">
-        <v>0</v>
-      </c>
-      <c r="T182" t="inlineStr">
-        <is>
-          <t>brain_coverage_pct:missing_fmriprep_brain_mask;tedana_rejected_components:missing_tedana_metrics</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="U182" t="inlineStr">
         <is>
-          <t>incomplete</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="V182" t="inlineStr">
@@ -17071,6 +17087,16 @@
       <c r="W182" t="inlineStr">
         <is>
           <t>derivatives/mriqc/sub-10929/ses-01/func/sub-10929_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
+        </is>
+      </c>
+      <c r="X182" t="inlineStr">
+        <is>
+          <t>derivatives/tedana/sub-10929/ses-01/sub-10929_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
+        </is>
+      </c>
+      <c r="Y182" t="inlineStr">
+        <is>
+          <t>derivatives/fmriprep/sub-10929/ses-01/func/sub-10929_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
@@ -17106,26 +17132,42 @@
       <c r="G183" t="n">
         <v>0.1676557362458465</v>
       </c>
+      <c r="H183" t="n">
+        <v>18</v>
+      </c>
+      <c r="I183" t="n">
+        <v>10</v>
+      </c>
+      <c r="J183" t="n">
+        <v>8</v>
+      </c>
+      <c r="K183" t="n">
+        <v>0.4444444444444444</v>
+      </c>
+      <c r="L183" t="n">
+        <v>99.97874488548807</v>
+      </c>
       <c r="M183" t="b">
         <v>0</v>
       </c>
       <c r="N183" t="b">
         <v>0</v>
       </c>
+      <c r="O183" t="b">
+        <v>0</v>
+      </c>
+      <c r="P183" t="b">
+        <v>0</v>
+      </c>
       <c r="Q183" t="b">
         <v>0</v>
       </c>
       <c r="S183" t="b">
-        <v>0</v>
-      </c>
-      <c r="T183" t="inlineStr">
-        <is>
-          <t>brain_coverage_pct:missing_fmriprep_brain_mask;tedana_rejected_components:missing_tedana_metrics</t>
-        </is>
+        <v>1</v>
       </c>
       <c r="U183" t="inlineStr">
         <is>
-          <t>incomplete</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="V183" t="inlineStr">
@@ -17136,6 +17178,16 @@
       <c r="W183" t="inlineStr">
         <is>
           <t>derivatives/mriqc/sub-10929/ses-01/func/sub-10929_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
+        </is>
+      </c>
+      <c r="X183" t="inlineStr">
+        <is>
+          <t>derivatives/tedana/sub-10929/ses-01/sub-10929_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
+        </is>
+      </c>
+      <c r="Y183" t="inlineStr">
+        <is>
+          <t>derivatives/fmriprep/sub-10929/ses-01/func/sub-10929_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
@@ -24696,7 +24748,7 @@
         <v>0.44</v>
       </c>
       <c r="L266" t="n">
-        <v>99.85387108773048</v>
+        <v>99.83792975184654</v>
       </c>
       <c r="M266" t="b">
         <v>0</v>
@@ -24787,7 +24839,7 @@
         <v>0.1379310344827586</v>
       </c>
       <c r="L267" t="n">
-        <v>99.79674796747967</v>
+        <v>99.75955151708379</v>
       </c>
       <c r="M267" t="b">
         <v>0</v>
@@ -24878,7 +24930,7 @@
         <v>0.2162162162162162</v>
       </c>
       <c r="L268" t="n">
-        <v>99.48987725171369</v>
+        <v>99.44603857803284</v>
       </c>
       <c r="M268" t="b">
         <v>0</v>
@@ -24969,7 +25021,7 @@
         <v>0.2142857142857143</v>
       </c>
       <c r="L269" t="n">
-        <v>99.90302354003933</v>
+        <v>99.89106753812636</v>
       </c>
       <c r="M269" t="b">
         <v>0</v>
@@ -25060,7 +25112,7 @@
         <v>0.3666666666666666</v>
       </c>
       <c r="L270" t="n">
-        <v>99.89106753812636</v>
+        <v>99.8791115362134</v>
       </c>
       <c r="M270" t="b">
         <v>0</v>
@@ -53177,14 +53229,14 @@
         <v>1</v>
       </c>
       <c r="P575" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q575" t="b">
         <v>1</v>
       </c>
       <c r="R575" t="inlineStr">
         <is>
-          <t>high_tedana_rejected_components</t>
+          <t>high_tedana_rejected_components;low_brain_coverage</t>
         </is>
       </c>
       <c r="S575" t="b">
@@ -54373,7 +54425,7 @@
         <v>0.8235294117647058</v>
       </c>
       <c r="L588" t="n">
-        <v>99.73458173282117</v>
+        <v>99.76220840639779</v>
       </c>
       <c r="M588" t="b">
         <v>0</v>
@@ -58659,7 +58711,7 @@
         <v>0.6984126984126984</v>
       </c>
       <c r="L634" t="n">
-        <v>99.71324157063594</v>
+        <v>99.73563951325788</v>
       </c>
       <c r="M634" t="b">
         <v>0</v>
@@ -58755,7 +58807,7 @@
         <v>0.7115384615384616</v>
       </c>
       <c r="L635" t="n">
-        <v>99.72257789159198</v>
+        <v>99.74228173654285</v>
       </c>
       <c r="M635" t="b">
         <v>0</v>
@@ -58809,7 +58861,7 @@
     <row r="636">
       <c r="A636" t="inlineStr">
         <is>
-          <t>12020</t>
+          <t>12018</t>
         </is>
       </c>
       <c r="B636" t="inlineStr">
@@ -58833,25 +58885,25 @@
         </is>
       </c>
       <c r="F636" t="n">
-        <v>62.08552327007055</v>
+        <v>42.28498629806563</v>
       </c>
       <c r="G636" t="n">
-        <v>0.09960429796200085</v>
+        <v>0.2484859609011503</v>
       </c>
       <c r="H636" t="n">
-        <v>29</v>
+        <v>42</v>
       </c>
       <c r="I636" t="n">
-        <v>8</v>
+        <v>19</v>
       </c>
       <c r="J636" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="K636" t="n">
-        <v>0.7241379310344828</v>
+        <v>0.5476190476190477</v>
       </c>
       <c r="L636" t="n">
-        <v>99.17636431266274</v>
+        <v>99.95748977097614</v>
       </c>
       <c r="M636" t="b">
         <v>0</v>
@@ -58878,29 +58930,29 @@
       </c>
       <c r="V636" t="inlineStr">
         <is>
-          <t>bids/sub-12020/ses-01/func/sub-12020_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12018/ses-01/func/sub-12018_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W636" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12020/ses-01/func/sub-12020_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12018/ses-01/func/sub-12018_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X636" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12020/ses-01/sub-12020_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12018/ses-01/sub-12018_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y636" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12020/ses-01/func/sub-12020_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12018/ses-01/func/sub-12018_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="637">
       <c r="A637" t="inlineStr">
         <is>
-          <t>12020</t>
+          <t>12018</t>
         </is>
       </c>
       <c r="B637" t="inlineStr">
@@ -58924,25 +58976,25 @@
         </is>
       </c>
       <c r="F637" t="n">
-        <v>60.43486697878689</v>
+        <v>45.42989409063011</v>
       </c>
       <c r="G637" t="n">
-        <v>0.09675230037304278</v>
+        <v>0.2412756131022805</v>
       </c>
       <c r="H637" t="n">
-        <v>31</v>
+        <v>41</v>
       </c>
       <c r="I637" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="J637" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="K637" t="n">
-        <v>0.5806451612903226</v>
+        <v>0.4878048780487805</v>
       </c>
       <c r="L637" t="n">
-        <v>99.13518252829587</v>
+        <v>99.98937244274404</v>
       </c>
       <c r="M637" t="b">
         <v>0</v>
@@ -58954,49 +59006,44 @@
         <v>0</v>
       </c>
       <c r="P637" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q637" t="b">
-        <v>1</v>
-      </c>
-      <c r="R637" t="inlineStr">
-        <is>
-          <t>low_brain_coverage</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="S637" t="b">
         <v>1</v>
       </c>
       <c r="U637" t="inlineStr">
         <is>
-          <t>outlier</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="V637" t="inlineStr">
         <is>
-          <t>bids/sub-12020/ses-01/func/sub-12020_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12018/ses-01/func/sub-12018_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W637" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12020/ses-01/func/sub-12020_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12018/ses-01/func/sub-12018_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X637" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12020/ses-01/sub-12020_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12018/ses-01/sub-12018_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y637" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12020/ses-01/func/sub-12020_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12018/ses-01/func/sub-12018_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="638">
       <c r="A638" t="inlineStr">
         <is>
-          <t>12021</t>
+          <t>12020</t>
         </is>
       </c>
       <c r="B638" t="inlineStr">
@@ -59020,25 +59067,25 @@
         </is>
       </c>
       <c r="F638" t="n">
-        <v>30.76991240610369</v>
+        <v>62.08552327007055</v>
       </c>
       <c r="G638" t="n">
-        <v>0.2196402911535911</v>
+        <v>0.09960429796200085</v>
       </c>
       <c r="H638" t="n">
-        <v>106</v>
+        <v>29</v>
       </c>
       <c r="I638" t="n">
-        <v>19</v>
+        <v>8</v>
       </c>
       <c r="J638" t="n">
-        <v>87</v>
+        <v>21</v>
       </c>
       <c r="K638" t="n">
-        <v>0.8207547169811321</v>
+        <v>0.7241379310344828</v>
       </c>
       <c r="L638" t="n">
-        <v>99.78744885488071</v>
+        <v>99.17636431266274</v>
       </c>
       <c r="M638" t="b">
         <v>0</v>
@@ -59047,52 +59094,47 @@
         <v>0</v>
       </c>
       <c r="O638" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P638" t="b">
         <v>0</v>
       </c>
       <c r="Q638" t="b">
-        <v>1</v>
-      </c>
-      <c r="R638" t="inlineStr">
-        <is>
-          <t>high_tedana_rejected_components</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="S638" t="b">
         <v>1</v>
       </c>
       <c r="U638" t="inlineStr">
         <is>
-          <t>outlier</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="V638" t="inlineStr">
         <is>
-          <t>bids/sub-12021/ses-01/func/sub-12021_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12020/ses-01/func/sub-12020_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W638" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12021/ses-01/func/sub-12021_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12020/ses-01/func/sub-12020_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X638" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12021/ses-01/sub-12021_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12020/ses-01/sub-12020_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y638" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12021/ses-01/func/sub-12021_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12020/ses-01/func/sub-12020_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="639">
       <c r="A639" t="inlineStr">
         <is>
-          <t>12021</t>
+          <t>12020</t>
         </is>
       </c>
       <c r="B639" t="inlineStr">
@@ -59116,25 +59158,25 @@
         </is>
       </c>
       <c r="F639" t="n">
-        <v>32.73531654849648</v>
+        <v>60.43486697878689</v>
       </c>
       <c r="G639" t="n">
-        <v>0.21809310482747</v>
+        <v>0.09675230037304278</v>
       </c>
       <c r="H639" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="I639" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="J639" t="n">
-        <v>21</v>
+        <v>18</v>
       </c>
       <c r="K639" t="n">
-        <v>0.6363636363636364</v>
+        <v>0.5806451612903226</v>
       </c>
       <c r="L639" t="n">
-        <v>99.74361018119986</v>
+        <v>99.13518252829587</v>
       </c>
       <c r="M639" t="b">
         <v>0</v>
@@ -59146,44 +59188,49 @@
         <v>0</v>
       </c>
       <c r="P639" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q639" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="R639" t="inlineStr">
+        <is>
+          <t>low_brain_coverage</t>
+        </is>
       </c>
       <c r="S639" t="b">
         <v>1</v>
       </c>
       <c r="U639" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>outlier</t>
         </is>
       </c>
       <c r="V639" t="inlineStr">
         <is>
-          <t>bids/sub-12021/ses-01/func/sub-12021_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12020/ses-01/func/sub-12020_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W639" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12021/ses-01/func/sub-12021_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12020/ses-01/func/sub-12020_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X639" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12021/ses-01/sub-12021_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12020/ses-01/sub-12020_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y639" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12021/ses-01/func/sub-12021_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12020/ses-01/func/sub-12020_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="640">
       <c r="A640" t="inlineStr">
         <is>
-          <t>12031</t>
+          <t>12021</t>
         </is>
       </c>
       <c r="B640" t="inlineStr">
@@ -59207,25 +59254,25 @@
         </is>
       </c>
       <c r="F640" t="n">
-        <v>44.18728492315859</v>
+        <v>30.76991240610369</v>
       </c>
       <c r="G640" t="n">
-        <v>0.1263781875021193</v>
+        <v>0.2196402911535911</v>
       </c>
       <c r="H640" t="n">
-        <v>45</v>
+        <v>106</v>
       </c>
       <c r="I640" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="J640" t="n">
-        <v>29</v>
+        <v>87</v>
       </c>
       <c r="K640" t="n">
-        <v>0.6444444444444445</v>
+        <v>0.8207547169811321</v>
       </c>
       <c r="L640" t="n">
-        <v>99.54832881662151</v>
+        <v>99.78744885488071</v>
       </c>
       <c r="M640" t="b">
         <v>0</v>
@@ -59234,47 +59281,52 @@
         <v>0</v>
       </c>
       <c r="O640" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P640" t="b">
         <v>0</v>
       </c>
       <c r="Q640" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="R640" t="inlineStr">
+        <is>
+          <t>high_tedana_rejected_components</t>
+        </is>
       </c>
       <c r="S640" t="b">
         <v>1</v>
       </c>
       <c r="U640" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>outlier</t>
         </is>
       </c>
       <c r="V640" t="inlineStr">
         <is>
-          <t>bids/sub-12031/ses-01/func/sub-12031_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12021/ses-01/func/sub-12021_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W640" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12031/ses-01/func/sub-12031_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12021/ses-01/func/sub-12021_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X640" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12031/ses-01/sub-12031_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12021/ses-01/sub-12021_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y640" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12031/ses-01/func/sub-12031_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12021/ses-01/func/sub-12021_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="641">
       <c r="A641" t="inlineStr">
         <is>
-          <t>12031</t>
+          <t>12021</t>
         </is>
       </c>
       <c r="B641" t="inlineStr">
@@ -59298,25 +59350,25 @@
         </is>
       </c>
       <c r="F641" t="n">
-        <v>49.70353406842332</v>
+        <v>32.73531654849648</v>
       </c>
       <c r="G641" t="n">
-        <v>0.1088629148394633</v>
+        <v>0.21809310482747</v>
       </c>
       <c r="H641" t="n">
-        <v>40</v>
+        <v>33</v>
       </c>
       <c r="I641" t="n">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="J641" t="n">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="K641" t="n">
-        <v>0.625</v>
+        <v>0.6363636363636364</v>
       </c>
       <c r="L641" t="n">
-        <v>99.84590041978851</v>
+        <v>99.74361018119986</v>
       </c>
       <c r="M641" t="b">
         <v>0</v>
@@ -59343,29 +59395,29 @@
       </c>
       <c r="V641" t="inlineStr">
         <is>
-          <t>bids/sub-12031/ses-01/func/sub-12031_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12021/ses-01/func/sub-12021_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W641" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12031/ses-01/func/sub-12031_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12021/ses-01/func/sub-12021_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X641" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12031/ses-01/sub-12031_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12021/ses-01/sub-12021_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y641" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12031/ses-01/func/sub-12031_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12021/ses-01/func/sub-12021_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="642">
       <c r="A642" t="inlineStr">
         <is>
-          <t>12033</t>
+          <t>12031</t>
         </is>
       </c>
       <c r="B642" t="inlineStr">
@@ -59389,25 +59441,25 @@
         </is>
       </c>
       <c r="F642" t="n">
-        <v>45.6717341565527</v>
+        <v>44.18728492315859</v>
       </c>
       <c r="G642" t="n">
-        <v>0.169422742780033</v>
+        <v>0.1263781875021193</v>
       </c>
       <c r="H642" t="n">
-        <v>37</v>
+        <v>45</v>
       </c>
       <c r="I642" t="n">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="J642" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
       <c r="K642" t="n">
-        <v>0.6756756756756757</v>
+        <v>0.6444444444444445</v>
       </c>
       <c r="L642" t="n">
-        <v>99.92826398852223</v>
+        <v>99.54832881662151</v>
       </c>
       <c r="M642" t="b">
         <v>0</v>
@@ -59434,29 +59486,29 @@
       </c>
       <c r="V642" t="inlineStr">
         <is>
-          <t>bids/sub-12033/ses-01/func/sub-12033_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12031/ses-01/func/sub-12031_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W642" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12033/ses-01/func/sub-12033_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12031/ses-01/func/sub-12031_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X642" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12033/ses-01/sub-12033_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12031/ses-01/sub-12031_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y642" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12033/ses-01/func/sub-12033_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12031/ses-01/func/sub-12031_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="643">
       <c r="A643" t="inlineStr">
         <is>
-          <t>12033</t>
+          <t>12031</t>
         </is>
       </c>
       <c r="B643" t="inlineStr">
@@ -59480,25 +59532,25 @@
         </is>
       </c>
       <c r="F643" t="n">
-        <v>46.6732823610073</v>
+        <v>49.70353406842332</v>
       </c>
       <c r="G643" t="n">
-        <v>0.1702473006721096</v>
+        <v>0.1088629148394633</v>
       </c>
       <c r="H643" t="n">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="I643" t="n">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="J643" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="K643" t="n">
-        <v>0.7027027027027027</v>
+        <v>0.625</v>
       </c>
       <c r="L643" t="n">
-        <v>99.90833731866731</v>
+        <v>99.84590041978851</v>
       </c>
       <c r="M643" t="b">
         <v>0</v>
@@ -59525,29 +59577,29 @@
       </c>
       <c r="V643" t="inlineStr">
         <is>
-          <t>bids/sub-12033/ses-01/func/sub-12033_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12031/ses-01/func/sub-12031_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W643" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12033/ses-01/func/sub-12033_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12031/ses-01/func/sub-12031_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X643" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12033/ses-01/sub-12033_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12031/ses-01/sub-12031_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y643" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12033/ses-01/func/sub-12033_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12031/ses-01/func/sub-12031_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="644">
       <c r="A644" t="inlineStr">
         <is>
-          <t>12036</t>
+          <t>12033</t>
         </is>
       </c>
       <c r="B644" t="inlineStr">
@@ -59571,25 +59623,25 @@
         </is>
       </c>
       <c r="F644" t="n">
-        <v>44.78085682913661</v>
+        <v>45.6717341565527</v>
       </c>
       <c r="G644" t="n">
-        <v>0.2014055375396319</v>
+        <v>0.169422742780033</v>
       </c>
       <c r="H644" t="n">
-        <v>53</v>
+        <v>37</v>
       </c>
       <c r="I644" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="J644" t="n">
-        <v>37</v>
+        <v>25</v>
       </c>
       <c r="K644" t="n">
-        <v>0.6981132075471698</v>
+        <v>0.6756756756756757</v>
       </c>
       <c r="L644" t="n">
-        <v>99.52175992348158</v>
+        <v>99.92826398852223</v>
       </c>
       <c r="M644" t="b">
         <v>0</v>
@@ -59598,52 +59650,47 @@
         <v>0</v>
       </c>
       <c r="O644" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P644" t="b">
         <v>0</v>
       </c>
       <c r="Q644" t="b">
-        <v>1</v>
-      </c>
-      <c r="R644" t="inlineStr">
-        <is>
-          <t>high_tedana_rejected_components</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="S644" t="b">
         <v>1</v>
       </c>
       <c r="U644" t="inlineStr">
         <is>
-          <t>outlier</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="V644" t="inlineStr">
         <is>
-          <t>bids/sub-12036/ses-01/func/sub-12036_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12033/ses-01/func/sub-12033_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W644" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12036/ses-01/func/sub-12036_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12033/ses-01/func/sub-12033_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X644" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12036/ses-01/sub-12036_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12033/ses-01/sub-12033_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y644" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12036/ses-01/func/sub-12036_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12033/ses-01/func/sub-12033_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="645">
       <c r="A645" t="inlineStr">
         <is>
-          <t>12036</t>
+          <t>12033</t>
         </is>
       </c>
       <c r="B645" t="inlineStr">
@@ -59667,25 +59714,25 @@
         </is>
       </c>
       <c r="F645" t="n">
-        <v>32.4732759273611</v>
+        <v>46.6732823610073</v>
       </c>
       <c r="G645" t="n">
-        <v>0.1820007202070183</v>
+        <v>0.1702473006721096</v>
       </c>
       <c r="H645" t="n">
-        <v>44</v>
+        <v>37</v>
       </c>
       <c r="I645" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="J645" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="K645" t="n">
-        <v>0.7727272727272727</v>
+        <v>0.7027027027027027</v>
       </c>
       <c r="L645" t="n">
-        <v>99.57356926510441</v>
+        <v>99.90833731866731</v>
       </c>
       <c r="M645" t="b">
         <v>0</v>
@@ -59712,29 +59759,29 @@
       </c>
       <c r="V645" t="inlineStr">
         <is>
-          <t>bids/sub-12036/ses-01/func/sub-12036_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12033/ses-01/func/sub-12033_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W645" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12036/ses-01/func/sub-12036_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12033/ses-01/func/sub-12033_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X645" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12036/ses-01/sub-12036_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12033/ses-01/sub-12033_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y645" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12036/ses-01/func/sub-12036_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12033/ses-01/func/sub-12033_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="646">
       <c r="A646" t="inlineStr">
         <is>
-          <t>12037</t>
+          <t>12036</t>
         </is>
       </c>
       <c r="B646" t="inlineStr">
@@ -59758,25 +59805,25 @@
         </is>
       </c>
       <c r="F646" t="n">
-        <v>57.21695437585004</v>
+        <v>44.78085682913661</v>
       </c>
       <c r="G646" t="n">
-        <v>0.1005715395521443</v>
+        <v>0.2014055375396319</v>
       </c>
       <c r="H646" t="n">
-        <v>46</v>
+        <v>53</v>
       </c>
       <c r="I646" t="n">
-        <v>28</v>
+        <v>16</v>
       </c>
       <c r="J646" t="n">
-        <v>18</v>
+        <v>37</v>
       </c>
       <c r="K646" t="n">
-        <v>0.391304347826087</v>
+        <v>0.6981132075471698</v>
       </c>
       <c r="L646" t="n">
-        <v>99.47924969445774</v>
+        <v>99.52175992348158</v>
       </c>
       <c r="M646" t="b">
         <v>0</v>
@@ -59785,47 +59832,52 @@
         <v>0</v>
       </c>
       <c r="O646" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P646" t="b">
         <v>0</v>
       </c>
       <c r="Q646" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="R646" t="inlineStr">
+        <is>
+          <t>high_tedana_rejected_components</t>
+        </is>
       </c>
       <c r="S646" t="b">
         <v>1</v>
       </c>
       <c r="U646" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>outlier</t>
         </is>
       </c>
       <c r="V646" t="inlineStr">
         <is>
-          <t>bids/sub-12037/ses-01/func/sub-12037_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12036/ses-01/func/sub-12036_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W646" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12037/ses-01/func/sub-12037_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12036/ses-01/func/sub-12036_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X646" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12037/ses-01/sub-12037_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12036/ses-01/sub-12036_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y646" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12037/ses-01/func/sub-12037_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12036/ses-01/func/sub-12036_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="647">
       <c r="A647" t="inlineStr">
         <is>
-          <t>12037</t>
+          <t>12036</t>
         </is>
       </c>
       <c r="B647" t="inlineStr">
@@ -59849,25 +59901,25 @@
         </is>
       </c>
       <c r="F647" t="n">
-        <v>56.46135326754302</v>
+        <v>32.4732759273611</v>
       </c>
       <c r="G647" t="n">
-        <v>0.1043699908217318</v>
+        <v>0.1820007202070183</v>
       </c>
       <c r="H647" t="n">
-        <v>20</v>
+        <v>44</v>
       </c>
       <c r="I647" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="J647" t="n">
-        <v>8</v>
+        <v>34</v>
       </c>
       <c r="K647" t="n">
-        <v>0.4</v>
+        <v>0.7727272727272727</v>
       </c>
       <c r="L647" t="n">
-        <v>99.38625856846804</v>
+        <v>99.57356926510441</v>
       </c>
       <c r="M647" t="b">
         <v>0</v>
@@ -59894,29 +59946,29 @@
       </c>
       <c r="V647" t="inlineStr">
         <is>
-          <t>bids/sub-12037/ses-01/func/sub-12037_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12036/ses-01/func/sub-12036_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W647" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12037/ses-01/func/sub-12037_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12036/ses-01/func/sub-12036_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X647" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12037/ses-01/sub-12037_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12036/ses-01/sub-12036_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y647" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12037/ses-01/func/sub-12037_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12036/ses-01/func/sub-12036_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="648">
       <c r="A648" t="inlineStr">
         <is>
-          <t>12038</t>
+          <t>12037</t>
         </is>
       </c>
       <c r="B648" t="inlineStr">
@@ -59940,25 +59992,25 @@
         </is>
       </c>
       <c r="F648" t="n">
-        <v>57.85016420576721</v>
+        <v>57.21695437585004</v>
       </c>
       <c r="G648" t="n">
-        <v>0.08639868741754726</v>
+        <v>0.1005715395521443</v>
       </c>
       <c r="H648" t="n">
-        <v>24</v>
+        <v>46</v>
       </c>
       <c r="I648" t="n">
-        <v>16</v>
+        <v>28</v>
       </c>
       <c r="J648" t="n">
-        <v>8</v>
+        <v>18</v>
       </c>
       <c r="K648" t="n">
-        <v>0.3333333333333333</v>
+        <v>0.391304347826087</v>
       </c>
       <c r="L648" t="n">
-        <v>99.32249322493224</v>
+        <v>99.47924969445774</v>
       </c>
       <c r="M648" t="b">
         <v>0</v>
@@ -59985,29 +60037,29 @@
       </c>
       <c r="V648" t="inlineStr">
         <is>
-          <t>bids/sub-12038/ses-01/func/sub-12038_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12037/ses-01/func/sub-12037_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W648" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12038/ses-01/func/sub-12038_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12037/ses-01/func/sub-12037_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X648" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12038/ses-01/sub-12038_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12037/ses-01/sub-12037_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y648" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12038/ses-01/func/sub-12038_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12037/ses-01/func/sub-12037_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="649">
       <c r="A649" t="inlineStr">
         <is>
-          <t>12038</t>
+          <t>12037</t>
         </is>
       </c>
       <c r="B649" t="inlineStr">
@@ -60031,25 +60083,25 @@
         </is>
       </c>
       <c r="F649" t="n">
-        <v>52.10025152983144</v>
+        <v>56.46135326754302</v>
       </c>
       <c r="G649" t="n">
-        <v>0.1066133861184249</v>
+        <v>0.1043699908217318</v>
       </c>
       <c r="H649" t="n">
-        <v>52</v>
+        <v>20</v>
       </c>
       <c r="I649" t="n">
-        <v>30</v>
+        <v>12</v>
       </c>
       <c r="J649" t="n">
-        <v>22</v>
+        <v>8</v>
       </c>
       <c r="K649" t="n">
-        <v>0.4230769230769231</v>
+        <v>0.4</v>
       </c>
       <c r="L649" t="n">
-        <v>99.39954301503799</v>
+        <v>99.38625856846804</v>
       </c>
       <c r="M649" t="b">
         <v>0</v>
@@ -60076,29 +60128,29 @@
       </c>
       <c r="V649" t="inlineStr">
         <is>
-          <t>bids/sub-12038/ses-01/func/sub-12038_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12037/ses-01/func/sub-12037_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W649" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12038/ses-01/func/sub-12038_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12037/ses-01/func/sub-12037_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X649" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12038/ses-01/sub-12038_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12037/ses-01/sub-12037_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y649" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12038/ses-01/func/sub-12038_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12037/ses-01/func/sub-12037_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="650">
       <c r="A650" t="inlineStr">
         <is>
-          <t>12039</t>
+          <t>12038</t>
         </is>
       </c>
       <c r="B650" t="inlineStr">
@@ -60122,25 +60174,25 @@
         </is>
       </c>
       <c r="F650" t="n">
-        <v>38.52442282624543</v>
+        <v>57.85016420576721</v>
       </c>
       <c r="G650" t="n">
-        <v>0.2513479265193468</v>
+        <v>0.08639868741754726</v>
       </c>
       <c r="H650" t="n">
-        <v>73</v>
+        <v>24</v>
       </c>
       <c r="I650" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="J650" t="n">
-        <v>50</v>
+        <v>8</v>
       </c>
       <c r="K650" t="n">
-        <v>0.684931506849315</v>
+        <v>0.3333333333333333</v>
       </c>
       <c r="L650" t="n">
-        <v>99.53238748073755</v>
+        <v>99.32249322493224</v>
       </c>
       <c r="M650" t="b">
         <v>0</v>
@@ -60149,52 +60201,47 @@
         <v>0</v>
       </c>
       <c r="O650" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P650" t="b">
         <v>0</v>
       </c>
       <c r="Q650" t="b">
-        <v>1</v>
-      </c>
-      <c r="R650" t="inlineStr">
-        <is>
-          <t>high_tedana_rejected_components</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="S650" t="b">
         <v>1</v>
       </c>
       <c r="U650" t="inlineStr">
         <is>
-          <t>outlier</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="V650" t="inlineStr">
         <is>
-          <t>bids/sub-12039/ses-01/func/sub-12039_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12038/ses-01/func/sub-12038_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W650" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12039/ses-01/func/sub-12039_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12038/ses-01/func/sub-12038_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X650" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12039/ses-01/sub-12039_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12038/ses-01/sub-12038_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y650" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12039/ses-01/func/sub-12039_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12038/ses-01/func/sub-12038_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="651">
       <c r="A651" t="inlineStr">
         <is>
-          <t>12039</t>
+          <t>12038</t>
         </is>
       </c>
       <c r="B651" t="inlineStr">
@@ -60218,25 +60265,25 @@
         </is>
       </c>
       <c r="F651" t="n">
-        <v>53.59258437878452</v>
+        <v>52.10025152983144</v>
       </c>
       <c r="G651" t="n">
-        <v>0.140284656113992</v>
+        <v>0.1066133861184249</v>
       </c>
       <c r="H651" t="n">
-        <v>34</v>
+        <v>52</v>
       </c>
       <c r="I651" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="J651" t="n">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="K651" t="n">
-        <v>0.5294117647058824</v>
+        <v>0.4230769230769231</v>
       </c>
       <c r="L651" t="n">
-        <v>99.63202083001222</v>
+        <v>99.39954301503799</v>
       </c>
       <c r="M651" t="b">
         <v>0</v>
@@ -60263,29 +60310,29 @@
       </c>
       <c r="V651" t="inlineStr">
         <is>
-          <t>bids/sub-12039/ses-01/func/sub-12039_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12038/ses-01/func/sub-12038_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W651" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12039/ses-01/func/sub-12039_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12038/ses-01/func/sub-12038_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X651" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12039/ses-01/sub-12039_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12038/ses-01/sub-12038_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y651" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12039/ses-01/func/sub-12039_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12038/ses-01/func/sub-12038_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="652">
       <c r="A652" t="inlineStr">
         <is>
-          <t>12041</t>
+          <t>12039</t>
         </is>
       </c>
       <c r="B652" t="inlineStr">
@@ -60309,25 +60356,25 @@
         </is>
       </c>
       <c r="F652" t="n">
-        <v>37.80872071394697</v>
+        <v>38.52442282624543</v>
       </c>
       <c r="G652" t="n">
-        <v>0.1687602715368111</v>
+        <v>0.2513479265193468</v>
       </c>
       <c r="H652" t="n">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="I652" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J652" t="n">
-        <v>54</v>
+        <v>50</v>
       </c>
       <c r="K652" t="n">
-        <v>0.72</v>
+        <v>0.684931506849315</v>
       </c>
       <c r="L652" t="n">
-        <v>99.42345501886392</v>
+        <v>99.53238748073755</v>
       </c>
       <c r="M652" t="b">
         <v>0</v>
@@ -60359,29 +60406,29 @@
       </c>
       <c r="V652" t="inlineStr">
         <is>
-          <t>bids/sub-12041/ses-01/func/sub-12041_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12039/ses-01/func/sub-12039_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W652" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12041/ses-01/func/sub-12041_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12039/ses-01/func/sub-12039_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X652" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12041/ses-01/sub-12041_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12039/ses-01/sub-12039_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y652" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12041/ses-01/func/sub-12041_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12039/ses-01/func/sub-12039_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="653">
       <c r="A653" t="inlineStr">
         <is>
-          <t>12047</t>
+          <t>12039</t>
         </is>
       </c>
       <c r="B653" t="inlineStr">
@@ -60401,29 +60448,29 @@
       </c>
       <c r="E653" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>2</t>
         </is>
       </c>
       <c r="F653" t="n">
-        <v>39.89033934398321</v>
+        <v>53.59258437878452</v>
       </c>
       <c r="G653" t="n">
-        <v>0.1143468449376623</v>
+        <v>0.140284656113992</v>
       </c>
       <c r="H653" t="n">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="I653" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="J653" t="n">
-        <v>23</v>
+        <v>18</v>
       </c>
       <c r="K653" t="n">
-        <v>0.6052631578947368</v>
+        <v>0.5294117647058824</v>
       </c>
       <c r="L653" t="n">
-        <v>99.38094478984006</v>
+        <v>99.63202083001222</v>
       </c>
       <c r="M653" t="b">
         <v>0</v>
@@ -60450,29 +60497,29 @@
       </c>
       <c r="V653" t="inlineStr">
         <is>
-          <t>bids/sub-12047/ses-01/func/sub-12047_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12039/ses-01/func/sub-12039_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W653" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12047/ses-01/func/sub-12047_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12039/ses-01/func/sub-12039_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X653" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12047/ses-01/sub-12047_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12039/ses-01/sub-12039_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y653" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12047/ses-01/func/sub-12047_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12039/ses-01/func/sub-12039_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="654">
       <c r="A654" t="inlineStr">
         <is>
-          <t>12047</t>
+          <t>12041</t>
         </is>
       </c>
       <c r="B654" t="inlineStr">
@@ -60492,29 +60539,29 @@
       </c>
       <c r="E654" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>1</t>
         </is>
       </c>
       <c r="F654" t="n">
-        <v>35.4770081298193</v>
+        <v>37.80872071394697</v>
       </c>
       <c r="G654" t="n">
-        <v>0.1178694971249013</v>
+        <v>0.1687602715368111</v>
       </c>
       <c r="H654" t="n">
-        <v>44</v>
+        <v>75</v>
       </c>
       <c r="I654" t="n">
         <v>21</v>
       </c>
       <c r="J654" t="n">
-        <v>23</v>
+        <v>54</v>
       </c>
       <c r="K654" t="n">
-        <v>0.5227272727272727</v>
+        <v>0.72</v>
       </c>
       <c r="L654" t="n">
-        <v>99.4261119081779</v>
+        <v>99.42345501886392</v>
       </c>
       <c r="M654" t="b">
         <v>0</v>
@@ -60523,47 +60570,52 @@
         <v>0</v>
       </c>
       <c r="O654" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="P654" t="b">
         <v>0</v>
       </c>
       <c r="Q654" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="R654" t="inlineStr">
+        <is>
+          <t>high_tedana_rejected_components</t>
+        </is>
       </c>
       <c r="S654" t="b">
         <v>1</v>
       </c>
       <c r="U654" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>outlier</t>
         </is>
       </c>
       <c r="V654" t="inlineStr">
         <is>
-          <t>bids/sub-12047/ses-01/func/sub-12047_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12041/ses-01/func/sub-12041_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W654" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12047/ses-01/func/sub-12047_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12041/ses-01/func/sub-12041_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X654" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12047/ses-01/sub-12047_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12041/ses-01/sub-12041_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y654" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12047/ses-01/func/sub-12047_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12041/ses-01/func/sub-12041_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="655">
       <c r="A655" t="inlineStr">
         <is>
-          <t>12049</t>
+          <t>12047</t>
         </is>
       </c>
       <c r="B655" t="inlineStr">
@@ -60587,25 +60639,25 @@
         </is>
       </c>
       <c r="F655" t="n">
-        <v>45.21797637059353</v>
+        <v>39.89033934398321</v>
       </c>
       <c r="G655" t="n">
-        <v>0.1624742898607847</v>
+        <v>0.1143468449376623</v>
       </c>
       <c r="H655" t="n">
-        <v>57</v>
+        <v>38</v>
       </c>
       <c r="I655" t="n">
+        <v>15</v>
+      </c>
+      <c r="J655" t="n">
         <v>23</v>
       </c>
-      <c r="J655" t="n">
-        <v>34</v>
-      </c>
       <c r="K655" t="n">
-        <v>0.5964912280701754</v>
+        <v>0.6052631578947368</v>
       </c>
       <c r="L655" t="n">
-        <v>99.61607949412827</v>
+        <v>99.38094478984006</v>
       </c>
       <c r="M655" t="b">
         <v>0</v>
@@ -60632,29 +60684,29 @@
       </c>
       <c r="V655" t="inlineStr">
         <is>
-          <t>bids/sub-12049/ses-01/func/sub-12049_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12047/ses-01/func/sub-12047_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W655" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12049/ses-01/func/sub-12049_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12047/ses-01/func/sub-12047_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X655" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12049/ses-01/sub-12049_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12047/ses-01/sub-12047_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y655" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12049/ses-01/func/sub-12049_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12047/ses-01/func/sub-12047_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="656">
       <c r="A656" t="inlineStr">
         <is>
-          <t>12049</t>
+          <t>12047</t>
         </is>
       </c>
       <c r="B656" t="inlineStr">
@@ -60678,25 +60730,25 @@
         </is>
       </c>
       <c r="F656" t="n">
-        <v>34.34538307227194</v>
+        <v>35.4770081298193</v>
       </c>
       <c r="G656" t="n">
-        <v>0.2955829073196637</v>
+        <v>0.1178694971249013</v>
       </c>
       <c r="H656" t="n">
-        <v>25</v>
+        <v>44</v>
       </c>
       <c r="I656" t="n">
-        <v>9</v>
+        <v>21</v>
       </c>
       <c r="J656" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="K656" t="n">
-        <v>0.64</v>
+        <v>0.5227272727272727</v>
       </c>
       <c r="L656" t="n">
-        <v>99.65061905521016</v>
+        <v>99.4261119081779</v>
       </c>
       <c r="M656" t="b">
         <v>0</v>
@@ -60723,29 +60775,29 @@
       </c>
       <c r="V656" t="inlineStr">
         <is>
-          <t>bids/sub-12049/ses-01/func/sub-12049_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12047/ses-01/func/sub-12047_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W656" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12049/ses-01/func/sub-12049_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12047/ses-01/func/sub-12047_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X656" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12049/ses-01/sub-12049_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12047/ses-01/sub-12047_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y656" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12049/ses-01/func/sub-12049_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12047/ses-01/func/sub-12047_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="657">
       <c r="A657" t="inlineStr">
         <is>
-          <t>12051</t>
+          <t>12049</t>
         </is>
       </c>
       <c r="B657" t="inlineStr">
@@ -60769,25 +60821,25 @@
         </is>
       </c>
       <c r="F657" t="n">
-        <v>58.79467609897256</v>
+        <v>45.21797637059353</v>
       </c>
       <c r="G657" t="n">
-        <v>0.121387112729465</v>
+        <v>0.1624742898607847</v>
       </c>
       <c r="H657" t="n">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="I657" t="n">
-        <v>17</v>
+        <v>23</v>
       </c>
       <c r="J657" t="n">
-        <v>26</v>
+        <v>34</v>
       </c>
       <c r="K657" t="n">
-        <v>0.6046511627906976</v>
+        <v>0.5964912280701754</v>
       </c>
       <c r="L657" t="n">
-        <v>99.73563951325788</v>
+        <v>99.61607949412827</v>
       </c>
       <c r="M657" t="b">
         <v>0</v>
@@ -60814,29 +60866,29 @@
       </c>
       <c r="V657" t="inlineStr">
         <is>
-          <t>bids/sub-12051/ses-01/func/sub-12051_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12049/ses-01/func/sub-12049_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W657" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12051/ses-01/func/sub-12051_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12049/ses-01/func/sub-12049_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X657" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12051/ses-01/sub-12051_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12049/ses-01/sub-12049_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y657" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12051/ses-01/func/sub-12051_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12049/ses-01/func/sub-12049_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="658">
       <c r="A658" t="inlineStr">
         <is>
-          <t>12051</t>
+          <t>12049</t>
         </is>
       </c>
       <c r="B658" t="inlineStr">
@@ -60860,25 +60912,25 @@
         </is>
       </c>
       <c r="F658" t="n">
-        <v>58.02577073161956</v>
+        <v>34.34538307227194</v>
       </c>
       <c r="G658" t="n">
-        <v>0.08688405388786562</v>
+        <v>0.2955829073196637</v>
       </c>
       <c r="H658" t="n">
-        <v>42</v>
+        <v>25</v>
       </c>
       <c r="I658" t="n">
-        <v>23</v>
+        <v>9</v>
       </c>
       <c r="J658" t="n">
-        <v>19</v>
+        <v>16</v>
       </c>
       <c r="K658" t="n">
-        <v>0.4523809523809524</v>
+        <v>0.64</v>
       </c>
       <c r="L658" t="n">
-        <v>99.75955151708379</v>
+        <v>99.65061905521016</v>
       </c>
       <c r="M658" t="b">
         <v>0</v>
@@ -60905,29 +60957,29 @@
       </c>
       <c r="V658" t="inlineStr">
         <is>
-          <t>bids/sub-12051/ses-01/func/sub-12051_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12049/ses-01/func/sub-12049_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W658" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12051/ses-01/func/sub-12051_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12049/ses-01/func/sub-12049_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X658" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12051/ses-01/sub-12051_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12049/ses-01/sub-12049_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y658" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12051/ses-01/func/sub-12051_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12049/ses-01/func/sub-12049_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="659">
       <c r="A659" t="inlineStr">
         <is>
-          <t>12054</t>
+          <t>12051</t>
         </is>
       </c>
       <c r="B659" t="inlineStr">
@@ -60951,25 +61003,25 @@
         </is>
       </c>
       <c r="F659" t="n">
-        <v>60.70757659338415</v>
+        <v>58.79467609897256</v>
       </c>
       <c r="G659" t="n">
-        <v>0.07867727084992221</v>
+        <v>0.121387112729465</v>
       </c>
       <c r="H659" t="n">
-        <v>29</v>
+        <v>43</v>
       </c>
       <c r="I659" t="n">
-        <v>13</v>
+        <v>17</v>
       </c>
       <c r="J659" t="n">
-        <v>16</v>
+        <v>26</v>
       </c>
       <c r="K659" t="n">
-        <v>0.5517241379310345</v>
+        <v>0.6046511627906976</v>
       </c>
       <c r="L659" t="n">
-        <v>98.76321802433711</v>
+        <v>99.73563951325788</v>
       </c>
       <c r="M659" t="b">
         <v>0</v>
@@ -60981,49 +61033,44 @@
         <v>0</v>
       </c>
       <c r="P659" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q659" t="b">
-        <v>1</v>
-      </c>
-      <c r="R659" t="inlineStr">
-        <is>
-          <t>low_brain_coverage</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="S659" t="b">
         <v>1</v>
       </c>
       <c r="U659" t="inlineStr">
         <is>
-          <t>outlier</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="V659" t="inlineStr">
         <is>
-          <t>bids/sub-12054/ses-01/func/sub-12054_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12051/ses-01/func/sub-12051_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W659" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12054/ses-01/func/sub-12054_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12051/ses-01/func/sub-12051_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X659" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12054/ses-01/sub-12054_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12051/ses-01/sub-12051_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y659" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12054/ses-01/func/sub-12054_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12051/ses-01/func/sub-12051_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="660">
       <c r="A660" t="inlineStr">
         <is>
-          <t>12054</t>
+          <t>12051</t>
         </is>
       </c>
       <c r="B660" t="inlineStr">
@@ -61047,25 +61094,25 @@
         </is>
       </c>
       <c r="F660" t="n">
-        <v>61.3161139478907</v>
+        <v>58.02577073161956</v>
       </c>
       <c r="G660" t="n">
-        <v>0.08175623833660248</v>
+        <v>0.08688405388786562</v>
       </c>
       <c r="H660" t="n">
-        <v>27</v>
+        <v>42</v>
       </c>
       <c r="I660" t="n">
-        <v>11</v>
+        <v>23</v>
       </c>
       <c r="J660" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="K660" t="n">
-        <v>0.5925925925925926</v>
+        <v>0.4523809523809524</v>
       </c>
       <c r="L660" t="n">
-        <v>98.68351134491738</v>
+        <v>99.75955151708379</v>
       </c>
       <c r="M660" t="b">
         <v>0</v>
@@ -61077,49 +61124,44 @@
         <v>0</v>
       </c>
       <c r="P660" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="Q660" t="b">
-        <v>1</v>
-      </c>
-      <c r="R660" t="inlineStr">
-        <is>
-          <t>low_brain_coverage</t>
-        </is>
+        <v>0</v>
       </c>
       <c r="S660" t="b">
         <v>1</v>
       </c>
       <c r="U660" t="inlineStr">
         <is>
-          <t>outlier</t>
+          <t>pass</t>
         </is>
       </c>
       <c r="V660" t="inlineStr">
         <is>
-          <t>bids/sub-12054/ses-01/func/sub-12054_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12051/ses-01/func/sub-12051_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W660" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12054/ses-01/func/sub-12054_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12051/ses-01/func/sub-12051_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X660" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12054/ses-01/sub-12054_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12051/ses-01/sub-12051_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y660" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12054/ses-01/func/sub-12054_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12051/ses-01/func/sub-12051_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="661">
       <c r="A661" t="inlineStr">
         <is>
-          <t>12055</t>
+          <t>12054</t>
         </is>
       </c>
       <c r="B661" t="inlineStr">
@@ -61143,25 +61185,25 @@
         </is>
       </c>
       <c r="F661" t="n">
-        <v>51.67674112552777</v>
+        <v>60.70757659338415</v>
       </c>
       <c r="G661" t="n">
-        <v>0.08752615631589676</v>
+        <v>0.07867727084992221</v>
       </c>
       <c r="H661" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
       <c r="I661" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="J661" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="K661" t="n">
-        <v>0.5416666666666666</v>
+        <v>0.5517241379310345</v>
       </c>
       <c r="L661" t="n">
-        <v>99.8206599713056</v>
+        <v>98.76321802433711</v>
       </c>
       <c r="M661" t="b">
         <v>0</v>
@@ -61173,44 +61215,49 @@
         <v>0</v>
       </c>
       <c r="P661" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q661" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="R661" t="inlineStr">
+        <is>
+          <t>low_brain_coverage</t>
+        </is>
       </c>
       <c r="S661" t="b">
         <v>1</v>
       </c>
       <c r="U661" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>outlier</t>
         </is>
       </c>
       <c r="V661" t="inlineStr">
         <is>
-          <t>bids/sub-12055/ses-01/func/sub-12055_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12054/ses-01/func/sub-12054_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W661" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12055/ses-01/func/sub-12055_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12054/ses-01/func/sub-12054_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X661" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12055/ses-01/sub-12055_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12054/ses-01/sub-12054_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y661" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12055/ses-01/func/sub-12055_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12054/ses-01/func/sub-12054_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="662">
       <c r="A662" t="inlineStr">
         <is>
-          <t>12055</t>
+          <t>12054</t>
         </is>
       </c>
       <c r="B662" t="inlineStr">
@@ -61234,25 +61281,25 @@
         </is>
       </c>
       <c r="F662" t="n">
-        <v>48.15898477239534</v>
+        <v>61.3161139478907</v>
       </c>
       <c r="G662" t="n">
-        <v>0.09547729277010625</v>
+        <v>0.08175623833660248</v>
       </c>
       <c r="H662" t="n">
-        <v>49</v>
+        <v>27</v>
       </c>
       <c r="I662" t="n">
-        <v>34</v>
+        <v>11</v>
       </c>
       <c r="J662" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="K662" t="n">
-        <v>0.3061224489795918</v>
+        <v>0.5925925925925926</v>
       </c>
       <c r="L662" t="n">
-        <v>99.7887772995377</v>
+        <v>98.68351134491738</v>
       </c>
       <c r="M662" t="b">
         <v>0</v>
@@ -61264,44 +61311,49 @@
         <v>0</v>
       </c>
       <c r="P662" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="Q662" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="R662" t="inlineStr">
+        <is>
+          <t>low_brain_coverage</t>
+        </is>
       </c>
       <c r="S662" t="b">
         <v>1</v>
       </c>
       <c r="U662" t="inlineStr">
         <is>
-          <t>pass</t>
+          <t>outlier</t>
         </is>
       </c>
       <c r="V662" t="inlineStr">
         <is>
-          <t>bids/sub-12055/ses-01/func/sub-12055_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12054/ses-01/func/sub-12054_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W662" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12055/ses-01/func/sub-12055_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12054/ses-01/func/sub-12054_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X662" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12055/ses-01/sub-12055_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12054/ses-01/sub-12054_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y662" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12055/ses-01/func/sub-12055_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12054/ses-01/func/sub-12054_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="663">
       <c r="A663" t="inlineStr">
         <is>
-          <t>12057</t>
+          <t>12055</t>
         </is>
       </c>
       <c r="B663" t="inlineStr">
@@ -61325,25 +61377,25 @@
         </is>
       </c>
       <c r="F663" t="n">
-        <v>76.01308403722942</v>
+        <v>51.67674112552777</v>
       </c>
       <c r="G663" t="n">
-        <v>0.06483193780260338</v>
+        <v>0.08752615631589676</v>
       </c>
       <c r="H663" t="n">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="I663" t="n">
-        <v>20</v>
+        <v>11</v>
       </c>
       <c r="J663" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="K663" t="n">
-        <v>0.4736842105263158</v>
+        <v>0.5416666666666666</v>
       </c>
       <c r="L663" t="n">
-        <v>99.3663318986131</v>
+        <v>99.8206599713056</v>
       </c>
       <c r="M663" t="b">
         <v>0</v>
@@ -61370,119 +61422,301 @@
       </c>
       <c r="V663" t="inlineStr">
         <is>
-          <t>bids/sub-12057/ses-01/func/sub-12057_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
+          <t>bids/sub-12055/ses-01/func/sub-12055_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
       <c r="W663" t="inlineStr">
         <is>
-          <t>derivatives/mriqc/sub-12057/ses-01/func/sub-12057_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
+          <t>derivatives/mriqc/sub-12055/ses-01/func/sub-12055_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
         </is>
       </c>
       <c r="X663" t="inlineStr">
         <is>
-          <t>derivatives/tedana/sub-12057/ses-01/sub-12057_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
+          <t>derivatives/tedana/sub-12055/ses-01/sub-12055_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
         </is>
       </c>
       <c r="Y663" t="inlineStr">
         <is>
-          <t>derivatives/fmriprep/sub-12057/ses-01/func/sub-12057_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+          <t>derivatives/fmriprep/sub-12055/ses-01/func/sub-12055_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
     <row r="664">
       <c r="A664" t="inlineStr">
         <is>
+          <t>12055</t>
+        </is>
+      </c>
+      <c r="B664" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C664" t="inlineStr">
+        <is>
+          <t>sharedreward</t>
+        </is>
+      </c>
+      <c r="D664" t="inlineStr">
+        <is>
+          <t>sharedreward</t>
+        </is>
+      </c>
+      <c r="E664" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="F664" t="n">
+        <v>48.15898477239534</v>
+      </c>
+      <c r="G664" t="n">
+        <v>0.09547729277010625</v>
+      </c>
+      <c r="H664" t="n">
+        <v>49</v>
+      </c>
+      <c r="I664" t="n">
+        <v>34</v>
+      </c>
+      <c r="J664" t="n">
+        <v>15</v>
+      </c>
+      <c r="K664" t="n">
+        <v>0.3061224489795918</v>
+      </c>
+      <c r="L664" t="n">
+        <v>99.7887772995377</v>
+      </c>
+      <c r="M664" t="b">
+        <v>0</v>
+      </c>
+      <c r="N664" t="b">
+        <v>0</v>
+      </c>
+      <c r="O664" t="b">
+        <v>0</v>
+      </c>
+      <c r="P664" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q664" t="b">
+        <v>0</v>
+      </c>
+      <c r="S664" t="b">
+        <v>1</v>
+      </c>
+      <c r="U664" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="V664" t="inlineStr">
+        <is>
+          <t>bids/sub-12055/ses-01/func/sub-12055_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
+        </is>
+      </c>
+      <c r="W664" t="inlineStr">
+        <is>
+          <t>derivatives/mriqc/sub-12055/ses-01/func/sub-12055_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
+        </is>
+      </c>
+      <c r="X664" t="inlineStr">
+        <is>
+          <t>derivatives/tedana/sub-12055/ses-01/sub-12055_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
+        </is>
+      </c>
+      <c r="Y664" t="inlineStr">
+        <is>
+          <t>derivatives/fmriprep/sub-12055/ses-01/func/sub-12055_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+        </is>
+      </c>
+    </row>
+    <row r="665">
+      <c r="A665" t="inlineStr">
+        <is>
           <t>12057</t>
         </is>
       </c>
-      <c r="B664" t="inlineStr">
-        <is>
-          <t>01</t>
-        </is>
-      </c>
-      <c r="C664" t="inlineStr">
-        <is>
-          <t>sharedreward</t>
-        </is>
-      </c>
-      <c r="D664" t="inlineStr">
-        <is>
-          <t>sharedreward</t>
-        </is>
-      </c>
-      <c r="E664" t="inlineStr">
+      <c r="B665" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C665" t="inlineStr">
+        <is>
+          <t>sharedreward</t>
+        </is>
+      </c>
+      <c r="D665" t="inlineStr">
+        <is>
+          <t>sharedreward</t>
+        </is>
+      </c>
+      <c r="E665" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="F665" t="n">
+        <v>76.01308403722942</v>
+      </c>
+      <c r="G665" t="n">
+        <v>0.06483193780260338</v>
+      </c>
+      <c r="H665" t="n">
+        <v>38</v>
+      </c>
+      <c r="I665" t="n">
+        <v>20</v>
+      </c>
+      <c r="J665" t="n">
+        <v>18</v>
+      </c>
+      <c r="K665" t="n">
+        <v>0.4736842105263158</v>
+      </c>
+      <c r="L665" t="n">
+        <v>99.3663318986131</v>
+      </c>
+      <c r="M665" t="b">
+        <v>0</v>
+      </c>
+      <c r="N665" t="b">
+        <v>0</v>
+      </c>
+      <c r="O665" t="b">
+        <v>0</v>
+      </c>
+      <c r="P665" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q665" t="b">
+        <v>0</v>
+      </c>
+      <c r="S665" t="b">
+        <v>1</v>
+      </c>
+      <c r="U665" t="inlineStr">
+        <is>
+          <t>pass</t>
+        </is>
+      </c>
+      <c r="V665" t="inlineStr">
+        <is>
+          <t>bids/sub-12057/ses-01/func/sub-12057_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.nii.gz</t>
+        </is>
+      </c>
+      <c r="W665" t="inlineStr">
+        <is>
+          <t>derivatives/mriqc/sub-12057/ses-01/func/sub-12057_ses-01_task-sharedreward_run-1_echo-2_part-mag_bold.json</t>
+        </is>
+      </c>
+      <c r="X665" t="inlineStr">
+        <is>
+          <t>derivatives/tedana/sub-12057/ses-01/sub-12057_ses-01_task-sharedreward_run-1_desc-tedana_metrics.tsv</t>
+        </is>
+      </c>
+      <c r="Y665" t="inlineStr">
+        <is>
+          <t>derivatives/fmriprep/sub-12057/ses-01/func/sub-12057_ses-01_task-sharedreward_run-1_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
+        </is>
+      </c>
+    </row>
+    <row r="666">
+      <c r="A666" t="inlineStr">
+        <is>
+          <t>12057</t>
+        </is>
+      </c>
+      <c r="B666" t="inlineStr">
+        <is>
+          <t>01</t>
+        </is>
+      </c>
+      <c r="C666" t="inlineStr">
+        <is>
+          <t>sharedreward</t>
+        </is>
+      </c>
+      <c r="D666" t="inlineStr">
+        <is>
+          <t>sharedreward</t>
+        </is>
+      </c>
+      <c r="E666" t="inlineStr">
         <is>
           <t>2</t>
         </is>
       </c>
-      <c r="F664" t="n">
+      <c r="F666" t="n">
         <v>76.58244009129703</v>
       </c>
-      <c r="G664" t="n">
+      <c r="G666" t="n">
         <v>0.06421566951458083</v>
       </c>
-      <c r="H664" t="n">
+      <c r="H666" t="n">
         <v>37</v>
       </c>
-      <c r="I664" t="n">
+      <c r="I666" t="n">
         <v>20</v>
       </c>
-      <c r="J664" t="n">
+      <c r="J666" t="n">
         <v>17</v>
       </c>
-      <c r="K664" t="n">
+      <c r="K666" t="n">
         <v>0.4594594594594595</v>
       </c>
-      <c r="L664" t="n">
+      <c r="L666" t="n">
         <v>99.4287687974919</v>
       </c>
-      <c r="M664" t="b">
-        <v>0</v>
-      </c>
-      <c r="N664" t="b">
-        <v>0</v>
-      </c>
-      <c r="O664" t="b">
-        <v>0</v>
-      </c>
-      <c r="P664" t="b">
-        <v>0</v>
-      </c>
-      <c r="Q664" t="b">
-        <v>0</v>
-      </c>
-      <c r="S664" t="b">
-        <v>1</v>
-      </c>
-      <c r="U664" t="inlineStr">
+      <c r="M666" t="b">
+        <v>0</v>
+      </c>
+      <c r="N666" t="b">
+        <v>0</v>
+      </c>
+      <c r="O666" t="b">
+        <v>0</v>
+      </c>
+      <c r="P666" t="b">
+        <v>0</v>
+      </c>
+      <c r="Q666" t="b">
+        <v>0</v>
+      </c>
+      <c r="S666" t="b">
+        <v>1</v>
+      </c>
+      <c r="U666" t="inlineStr">
         <is>
           <t>pass</t>
         </is>
       </c>
-      <c r="V664" t="inlineStr">
+      <c r="V666" t="inlineStr">
         <is>
           <t>bids/sub-12057/ses-01/func/sub-12057_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.nii.gz</t>
         </is>
       </c>
-      <c r="W664" t="inlineStr">
+      <c r="W666" t="inlineStr">
         <is>
           <t>derivatives/mriqc/sub-12057/ses-01/func/sub-12057_ses-01_task-sharedreward_run-2_echo-2_part-mag_bold.json</t>
         </is>
       </c>
-      <c r="X664" t="inlineStr">
+      <c r="X666" t="inlineStr">
         <is>
           <t>derivatives/tedana/sub-12057/ses-01/sub-12057_ses-01_task-sharedreward_run-2_desc-tedana_metrics.tsv</t>
         </is>
       </c>
-      <c r="Y664" t="inlineStr">
+      <c r="Y666" t="inlineStr">
         <is>
           <t>derivatives/fmriprep/sub-12057/ses-01/func/sub-12057_ses-01_task-sharedreward_run-2_part-mag_space-MNI152NLin6Asym_desc-brain_mask.nii.gz</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Y664"/>
-  <conditionalFormatting sqref="A2:Y664">
+  <autoFilter ref="A1:Y666"/>
+  <conditionalFormatting sqref="A2:Y666">
     <cfRule type="expression" priority="1" dxfId="0">
       <formula>$Q2=TRUE</formula>
     </cfRule>
@@ -61590,22 +61824,22 @@
         </is>
       </c>
       <c r="D2" t="n">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="E2" t="n">
-        <v>23.76983295241371</v>
+        <v>23.77489347476512</v>
       </c>
       <c r="F2" t="n">
-        <v>38.70523553696694</v>
+        <v>38.75234285066836</v>
       </c>
       <c r="G2" t="n">
-        <v>14.93540258455323</v>
+        <v>14.97744937590323</v>
       </c>
       <c r="H2" t="n">
-        <v>1.366729075583862</v>
+        <v>1.308719410910271</v>
       </c>
       <c r="I2" t="n">
-        <v>61.10833941379678</v>
+        <v>61.21851691452321</v>
       </c>
       <c r="J2" t="inlineStr">
         <is>
@@ -61633,22 +61867,22 @@
         </is>
       </c>
       <c r="D3" t="n">
-        <v>663</v>
+        <v>665</v>
       </c>
       <c r="E3" t="n">
-        <v>0.1183975286117984</v>
+        <v>0.1184968769408362</v>
       </c>
       <c r="F3" t="n">
-        <v>0.2393154477238457</v>
+        <v>0.2402382593821463</v>
       </c>
       <c r="G3" t="n">
-        <v>0.1209179191120473</v>
+        <v>0.1217413824413101</v>
       </c>
       <c r="H3" t="n">
-        <v>-0.06297935005627249</v>
+        <v>-0.06411519672112902</v>
       </c>
       <c r="I3" t="n">
-        <v>0.4206923263919167</v>
+        <v>0.4228503330441115</v>
       </c>
       <c r="J3" t="inlineStr">
         <is>
@@ -61676,7 +61910,7 @@
         </is>
       </c>
       <c r="D4" t="n">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="E4" t="n">
         <v>9</v>
@@ -61719,22 +61953,22 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>661</v>
+        <v>665</v>
       </c>
       <c r="E5" t="n">
-        <v>99.60412349221531</v>
+        <v>99.60545193687231</v>
       </c>
       <c r="F5" t="n">
-        <v>99.90435198469632</v>
+        <v>99.90568042935331</v>
       </c>
       <c r="G5" t="n">
-        <v>0.3002284924810112</v>
+        <v>0.300228492480997</v>
       </c>
       <c r="H5" t="n">
-        <v>99.15378075349379</v>
+        <v>99.15510919815083</v>
       </c>
       <c r="I5" t="n">
-        <v>100.3546947234178</v>
+        <v>100.3560231680748</v>
       </c>
       <c r="J5" t="inlineStr">
         <is>
@@ -61742,7 +61976,7 @@
         </is>
       </c>
       <c r="K5" t="n">
-        <v>31</v>
+        <v>32</v>
       </c>
     </row>
   </sheetData>

</xml_diff>